<commit_message>
price-check: 2026-09-21 (re-execução solicitada pelo usuário)
</commit_message>
<xml_diff>
--- a/price-check/daily/2026-09-21.xlsx
+++ b/price-check/daily/2026-09-21.xlsx
@@ -101,27 +101,27 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>68</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robô Aspirador Anker eufy X10 Pro 4 em 1 Sucção 8000Pa IA Evita Obstáculos Mapeamento AI.Map 3.0 Lava Seca Esvazia Reabastece Água Escovas Antiembaraço Navegação Laser Limpeza Silenciosa Ideal Pet220V</t>
+          <t xml:space="preserve">Extratora de Sujeira Portátil WAP Spot Cleaner W3 Borrifa Esfrega e Extrai 1450W de Potência e Bico de Autolimpeza</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Extratoras</t>
         </is>
       </c>
       <c r="D2">
-        <v>7999.0</v>
+        <v>1011.0</v>
       </c>
       <c r="E2">
-        <v>4849.0</v>
+        <v>489.28</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$7999.00 por R$4749.00</t>
+          <t xml:space="preserve">de R$1011.00 por R$526.11</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -138,11 +138,11 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>67</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robô De Limpeza Wap Robot W500 Policleaner</t>
+          <t xml:space="preserve">Dreame L40 Ultra Com Base E Mop 19000pa Branco 127v</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -151,14 +151,14 @@
         </is>
       </c>
       <c r="D3">
-        <v>1399.0</v>
+        <v>7499.0</v>
       </c>
       <c r="E3">
-        <v>800.91</v>
+        <v>6599.0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$1399.00 por R$782.91</t>
+          <t xml:space="preserve">de R$7499.00 por R$6599.00</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -175,27 +175,27 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>66</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robô Aspirador de Pó 3 em 1 – Varre Aspira e Passa Pano com Lds Mapeamento Lydsto R1D Compatível com XiaoMi Home</t>
+          <t xml:space="preserve">Aspirador Automotivo Portátil WAP CAR com Filtro HEPA e Cabo de 3,7m</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Portáteis</t>
         </is>
       </c>
       <c r="D4">
-        <v>3500.0</v>
+        <v>111.0</v>
       </c>
       <c r="E4">
-        <v>1217.7</v>
+        <v>99.9</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$3500.00 por R$1230.00</t>
+          <t xml:space="preserve">de R$111.00 por R$99.90</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -212,48 +212,48 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arno X-PERT 7.60 Aspirador Versátil Sem Fio Bateria Removível RH6A Bivolt</t>
+          <t xml:space="preserve">Aspirador de Pó e Água WAP GTW 10 1400W de Potência com Bocal de Sopro</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portáteis</t>
+          <t xml:space="preserve">Aspiradores</t>
         </is>
       </c>
       <c r="D5">
-        <v>719.28</v>
+        <v>485.57</v>
       </c>
       <c r="E5">
-        <v>698.99</v>
-      </c>
-      <c r="F5"/>
+        <v>257.9</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$485.57 por R$260.91</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H5"/>
       <c r="I5"/>
       <c r="J5">
-        <v>7</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">não encontrou âncora do produto (título/buy-box) na página Amazon</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K5"/>
     </row>
     <row r="6">
       <c r="A6">
-        <v>64</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arno X-FORCE FLEX 9.60 Aqua Aspirador Versátil Sem Fio com Tubo Flexível XF9A Bivolt</t>
+          <t xml:space="preserve">Aspirador Portátil 3 Em 1 Com Soprador e Filtro HEPA Para Carro e Teclado USB</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -262,220 +262,224 @@
         </is>
       </c>
       <c r="D6">
-        <v>1819.0</v>
+        <v>59.99</v>
       </c>
       <c r="E6">
-        <v>1249.99</v>
-      </c>
-      <c r="F6"/>
+        <v>39.99</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$59.99 por R$39.99</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H6"/>
       <c r="I6"/>
       <c r="J6">
-        <v>7</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K6"/>
     </row>
     <row r="7">
       <c r="A7">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arno X-CLEAN 4 Limpadora de Pisos Vertical Sem Fio 2 em 1 LXC4 Bivolt</t>
+          <t xml:space="preserve">Robô Aspirador De Pó Inteligente Passa Pano Mapeamento Ekaza Preto</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vertical</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D7">
-        <v>2849.04</v>
+        <v>999.0</v>
       </c>
       <c r="E7">
-        <v>2899.99</v>
-      </c>
-      <c r="F7"/>
+        <v>565.62</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$1999.00 por R$919.99</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
-        </is>
-      </c>
-      <c r="H7"/>
-      <c r="I7"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H7">
+        <v>1999.0</v>
+      </c>
+      <c r="I7">
+        <v>919.99</v>
+      </c>
       <c r="J7">
-        <v>4</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K7"/>
     </row>
     <row r="8">
       <c r="A8">
-        <v>62</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Velds Robô Aspirador V50 PRO Base Autolimpante Mop Duplo Giratório 10000Pa 127V</t>
+          <t xml:space="preserve">Aspirador De Pó Portátil 21v + Filtro Hepa Com Acessórios</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Portáteis</t>
         </is>
       </c>
       <c r="D8">
-        <v>2449.99</v>
+        <v>699.04</v>
       </c>
       <c r="E8">
-        <v>2327.49</v>
-      </c>
-      <c r="F8"/>
+        <v>289.9</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$699.04 por R$289.90</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H8"/>
       <c r="I8"/>
       <c r="J8">
-        <v>7</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K8"/>
     </row>
     <row r="9">
       <c r="A9">
-        <v>61</v>
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robô Aspirador de Pó X600 com Mapeamento a Laser 3000Pa e Passa Pano</t>
+          <t xml:space="preserve">Aspirador Vertical WAP POWER SPEED MAX CI10 3 EM 1 1600W 127V</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Vertical</t>
         </is>
       </c>
       <c r="D9">
-        <v>1048.19</v>
+        <v>359.9</v>
       </c>
       <c r="E9">
-        <v>1048.19</v>
-      </c>
-      <c r="F9"/>
+        <v>226.73</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$359.90 por R$237.90</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H9"/>
       <c r="I9"/>
       <c r="J9">
-        <v>1</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K9"/>
     </row>
     <row r="10">
       <c r="A10">
-        <v>60</v>
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips Walita Aspirador de Pó Vertical com Mop Série 3000 XC3133/01</t>
+          <t xml:space="preserve">Robô Aspirador Wap Robot W90 Varre, Aspira e Passa Pano 30W Preto</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vertical</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D10">
-        <v>1999.9</v>
+        <v>514.14</v>
       </c>
       <c r="E10">
-        <v>1329.91</v>
-      </c>
-      <c r="F10"/>
+        <v>359.9</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$514.14 por R$359.90</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H10"/>
       <c r="I10"/>
       <c r="J10">
-        <v>2</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K10"/>
     </row>
     <row r="11">
       <c r="A11">
-        <v>59</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Britânia Aspirador de Pó Vertical BAS1500V Filtro Ciclone 1500W 220V</t>
+          <t xml:space="preserve">Mini Aspirador De Pó Portátil Recarregável Chrome Technology Soprador Usb Automotivo 3em1 Sem Fio</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vertical</t>
+          <t xml:space="preserve">Portáteis</t>
         </is>
       </c>
       <c r="D11">
-        <v>249.0</v>
+        <v>59.99</v>
       </c>
       <c r="E11">
-        <v>153.49</v>
-      </c>
-      <c r="F11"/>
+        <v>39.98</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$59.99 por R$39.99</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H11"/>
       <c r="I11"/>
       <c r="J11">
-        <v>6</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K11"/>
     </row>
     <row r="12">
       <c r="A12">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrolux Aspirador de Pó Vertical Ergorapido 2 em 1 ERG24N 30min Bivolt</t>
+          <t xml:space="preserve">Aspirador de Pó Vertical e Portátil WAP High Speed Plus 1350W 3 em 1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -484,121 +488,125 @@
         </is>
       </c>
       <c r="D12">
-        <v>1099.99</v>
+        <v>326.0</v>
       </c>
       <c r="E12">
-        <v>759.0</v>
-      </c>
-      <c r="F12"/>
+        <v>164.99</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$326.00 por R$160.04</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H12"/>
       <c r="I12"/>
       <c r="J12">
-        <v>7</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K12"/>
     </row>
     <row r="13">
       <c r="A13">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mondial Aspirador de Pó Hepa Turbo AP-15 1500W 110V</t>
+          <t xml:space="preserve">Robô Aspirador WAP Robot W200 3 em 1 Varre, Aspira e Passa Pano Bivolt</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspiradores</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D13">
-        <v>439.9</v>
+        <v>699.9</v>
       </c>
       <c r="E13">
-        <v>246.05</v>
-      </c>
-      <c r="F13"/>
+        <v>559.0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$999.00 por R$565.62</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H13"/>
       <c r="I13"/>
       <c r="J13">
-        <v>7</v>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K13"/>
     </row>
     <row r="14">
       <c r="A14">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philco Aspirador Robô PAS23 3 em 1 com MOP Bivolt Anticolisão</t>
+          <t xml:space="preserve">WAP Aspirador de Pó e Água GTW INOX 20i, Compacto, 20 Litros, com Soprador e Filtro Lavável, 170mbar 1900W 220v</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Profissionais</t>
         </is>
       </c>
       <c r="D14">
-        <v>699.9</v>
+        <v>759.9</v>
       </c>
       <c r="E14">
-        <v>484.4</v>
-      </c>
-      <c r="F14"/>
+        <v>500.47</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$759.90 por R$548.99</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H14"/>
       <c r="I14"/>
       <c r="J14">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t xml:space="preserve">não encontrou âncora do produto (título/buy-box) na página Amazon</t>
+          <t xml:space="preserve">preço não encontrado na janela da âncora (provável renderização JS); preço resolvido via fallback Tavily</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrolux Aspirador de Pó Sem Saco Ease C4 EAS40 1600W Cyclonic Power Filtro HEPA 127V</t>
+          <t xml:space="preserve">Dreame X50 Ultra Robô Aspirador e Esfregão, 20.000Pa, supera obstáculos de 6 cm, mopa extensível e removível, navegação LDS inteligente, 127V</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspiradores</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D15">
-        <v>729.9</v>
+        <v>4749.0</v>
       </c>
       <c r="E15">
-        <v>539.9</v>
+        <v>4749.0</v>
       </c>
       <c r="F15"/>
       <c r="G15" t="inlineStr">
@@ -609,132 +617,132 @@
       <c r="H15"/>
       <c r="I15"/>
       <c r="J15">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); fallback Tavily tentado mas não encontrou preço confiável</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kärcher Aspirador WDL 1s 3 em 1 Pó, Água e Soprador 1700W Tanque Inox 110V</t>
+          <t xml:space="preserve">Robô Aspirador e Esfregão Combinado 3 em 1 com Sucção 6500Pa</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Profissionais</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D16">
-        <v>479.0</v>
+        <v>999.0</v>
       </c>
       <c r="E16">
-        <v>323.91</v>
-      </c>
-      <c r="F16"/>
+        <v>532.97</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$999.00 por R$517.00</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H16"/>
       <c r="I16"/>
       <c r="J16">
-        <v>7</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K16"/>
     </row>
     <row r="17">
       <c r="A17">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">WAP Robô Aspirador de Pó ROBOT W100 3 em 1, Automático, 250ml, Bivolt</t>
+          <t xml:space="preserve">Aspirador de Pó e Água Wap GTW Inox 12 1400W com Bocal de Sopro</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Aspiradores</t>
         </is>
       </c>
       <c r="D17">
-        <v>799.9</v>
+        <v>485.57</v>
       </c>
       <c r="E17">
-        <v>648.87</v>
-      </c>
-      <c r="F17"/>
+        <v>260.91</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$349.99 por R$284.05</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H17"/>
       <c r="I17"/>
       <c r="J17">
-        <v>7</v>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K17"/>
     </row>
     <row r="18">
       <c r="A18">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philco Aspirador de Pó Vertical Power Clean PAS4000V 2000W 220V</t>
+          <t xml:space="preserve">Robô Aspirador Xiaomi S40 10.000Pa Ultra Potente Bivolt Branco</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vertical</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D18">
-        <v>434.9</v>
+        <v>1209.0</v>
       </c>
       <c r="E18">
-        <v>234.99</v>
-      </c>
-      <c r="F18"/>
+        <v>1209.0</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$1188.00 por R$1104.00</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H18"/>
       <c r="I18"/>
       <c r="J18">
-        <v>7</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K18"/>
     </row>
     <row r="19">
       <c r="A19">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Midea Aspirador de Pó Vertical 2 em 1 1350W Preto e Azul 220V</t>
+          <t xml:space="preserve">Aspirador Vertical WAP Power Speed Max AZ20 1600W, Sistema 360° com Tecnologia Cyclone, 3 em 1, 127V</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -743,72 +751,76 @@
         </is>
       </c>
       <c r="D19">
-        <v>209.0</v>
+        <v>359.9</v>
       </c>
       <c r="E19">
-        <v>141.45</v>
-      </c>
-      <c r="F19"/>
+        <v>237.9</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$348.00 por R$319.90</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
-        </is>
-      </c>
-      <c r="H19"/>
-      <c r="I19"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H19">
+        <v>348.0</v>
+      </c>
+      <c r="I19">
+        <v>319.9</v>
+      </c>
       <c r="J19">
-        <v>7</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K19"/>
     </row>
     <row r="20">
       <c r="A20">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrolux Aspirador de Pó sem Saco Easybox Bocal Pet EAS41 1800W Filtro HEPA 220V</t>
+          <t xml:space="preserve">Robô Aspirador Liectroux T9 com Base Autolimpante, Aspira, Varre e Passa Pano, para Carpetes e Pelo de Animais</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspiradores</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D20">
-        <v>952.0</v>
+        <v>2899.0</v>
       </c>
       <c r="E20">
-        <v>661.93</v>
-      </c>
-      <c r="F20"/>
+        <v>2413.0</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$2899.00 por R$2413.00</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H20"/>
       <c r="I20"/>
       <c r="J20">
-        <v>6</v>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K20"/>
     </row>
     <row r="21">
       <c r="A21">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrolux Aspirador de Pó Vertical Ergorapido 2 em 1 ERG25N 38min Bivolt Azul</t>
+          <t xml:space="preserve">Britânia BAS1295P Aspirador de Pó 2 em 1 1250W Preto 127V</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -817,35 +829,35 @@
         </is>
       </c>
       <c r="D21">
-        <v>1299.0</v>
+        <v>185.36</v>
       </c>
       <c r="E21">
-        <v>759.9</v>
-      </c>
-      <c r="F21"/>
+        <v>129.9</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$185.36 por R$129.90</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H21"/>
       <c r="I21"/>
       <c r="J21">
-        <v>7</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K21"/>
     </row>
     <row r="22">
       <c r="A22">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kärcher Aspirador de Pó Vertical 2 em 1 VCL 2 com Filtro HEPA 127V</t>
+          <t xml:space="preserve">Aspirador de Pó Vertical e Portátil WAP High Speed Plus 1350W, Tecnologia Cyclone, Filtro HEPA, 3 em 1, Vermelho</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -854,257 +866,257 @@
         </is>
       </c>
       <c r="D22">
-        <v>399.0</v>
+        <v>207.0</v>
       </c>
       <c r="E22">
-        <v>224.91</v>
-      </c>
-      <c r="F22"/>
+        <v>144.53</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$299.90 por R$153.44</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H22"/>
       <c r="I22"/>
       <c r="J22">
-        <v>7</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K22"/>
     </row>
     <row r="23">
       <c r="A23">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó Philco PAS70 1800W 2,2L Super Silencioso com Filtro HEPA 127V</t>
+          <t xml:space="preserve">Aspirador de Pó Vertical Sem Fio 3 em 1 Oster OASP630</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspiradores</t>
+          <t xml:space="preserve">Vertical</t>
         </is>
       </c>
       <c r="D23">
-        <v>347.9</v>
+        <v>539.9</v>
       </c>
       <c r="E23">
-        <v>313.39</v>
-      </c>
-      <c r="F23"/>
+        <v>334.22</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$539.90 por R$334.22</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H23"/>
       <c r="I23"/>
       <c r="J23">
-        <v>7</v>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K23"/>
     </row>
     <row r="24">
       <c r="A24">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xiaomi Robô Aspirador de Pó Inteligente S40 Branco</t>
+          <t xml:space="preserve">Aspirador de Pelos Kärcher Pet Clean com Tosador Recarregável, Kit 5 em 1, 300W</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Portáteis</t>
         </is>
       </c>
       <c r="D24">
-        <v>1290.0</v>
+        <v>542.56</v>
       </c>
       <c r="E24">
-        <v>1220.0</v>
-      </c>
-      <c r="F24"/>
+        <v>542.56</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$749.00 por R$534.31</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H24"/>
       <c r="I24"/>
       <c r="J24">
-        <v>7</v>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">preço não encontrado perto do buy-box (pode exigir JS / fora de estoque)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K24"/>
     </row>
     <row r="25">
       <c r="A25">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xiaomi Robô Aspirador de Pó Inteligente S40C Branco</t>
+          <t xml:space="preserve">Mini Aspirador de Pó Betahome Portátil 120W, USB, Soprador, Sem Fio, 6000Pa</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Portáteis</t>
         </is>
       </c>
       <c r="D25">
-        <v>2699.99</v>
+        <v>61.76</v>
       </c>
       <c r="E25">
-        <v>1055.0</v>
-      </c>
-      <c r="F25"/>
+        <v>41.99</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$61.76 por R$41.99</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H25"/>
       <c r="I25"/>
       <c r="J25">
-        <v>7</v>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K25"/>
     </row>
     <row r="26">
       <c r="A26">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrolux Aspirador de Pó e Água A10N1 1400W 18L (11L útil) com Função Sopro 127V</t>
+          <t xml:space="preserve">Aspirador de Pó Mondial Turbo Cycle AP-36 1100W, 2 em 1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Profissionais</t>
+          <t xml:space="preserve">Vertical</t>
         </is>
       </c>
       <c r="D26">
-        <v>379.9</v>
+        <v>316.9</v>
       </c>
       <c r="E26">
-        <v>259.9</v>
-      </c>
-      <c r="F26"/>
+        <v>196.97</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$316.90 por R$196.97</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H26"/>
       <c r="I26"/>
       <c r="J26">
-        <v>7</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">preço não encontrado perto do buy-box (pode exigir JS / fora de estoque)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K26"/>
     </row>
     <row r="27">
       <c r="A27">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">WAP Aspirador de Pó e Água GTW Inox 70i 2800W com Autolimpeza e Bocal de Sopro 70 Litros 127V</t>
+          <t xml:space="preserve">Aspirador de Pó Sem Fio Arno X-Force Flex 9.60 RH20</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Profissionais</t>
+          <t xml:space="preserve">Vertical</t>
         </is>
       </c>
       <c r="D27">
-        <v>2099.9</v>
+        <v>1599.0</v>
       </c>
       <c r="E27">
-        <v>1994.9</v>
-      </c>
-      <c r="F27"/>
+        <v>1199.0</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$1499.00 por R$1199.00</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H27"/>
       <c r="I27"/>
       <c r="J27">
-        <v>7</v>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K27"/>
     </row>
     <row r="28">
       <c r="A28">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">WAP Robô Aspirador de Pó ROBOT W90 3 em 1, Automático, 250ml, Bivolt</t>
+          <t xml:space="preserve">Aspirador de Pó Mondial Turbo Cycle HEPA 1550W AP-41-GI</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Vertical</t>
         </is>
       </c>
       <c r="D28">
-        <v>359.9</v>
+        <v>329.9</v>
       </c>
       <c r="E28">
-        <v>315.76</v>
-      </c>
-      <c r="F28"/>
+        <v>235.47</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$329.90 por R$235.50</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H28"/>
       <c r="I28"/>
       <c r="J28">
-        <v>1</v>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">preço não encontrado perto do buy-box (pode exigir JS / fora de estoque)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K28"/>
     </row>
     <row r="29">
       <c r="A29">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">WAP Aspirador de Pó Vertical à Bateria Eco Rápido 2 em 1, 700ml, Bivolt</t>
+          <t xml:space="preserve">Aspirador de Pó Vertical 2 em 1 Philco PAS1550C 1400W</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1113,47 +1125,51 @@
         </is>
       </c>
       <c r="D29">
-        <v>959.9</v>
+        <v>206.9</v>
       </c>
       <c r="E29">
-        <v>499.9</v>
-      </c>
-      <c r="F29"/>
+        <v>159.82</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$206.90 por R$194.90</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
-        </is>
-      </c>
-      <c r="H29"/>
-      <c r="I29"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H29">
+        <v>206.9</v>
+      </c>
+      <c r="I29">
+        <v>194.9</v>
+      </c>
       <c r="J29">
-        <v>7</v>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K29"/>
     </row>
     <row r="30">
       <c r="A30">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Black+Decker Aspirador de Pó e Água Portátil à Bateria 3,6V APB3600 Vermelho Bivolt</t>
+          <t xml:space="preserve">Aspirador de Pó Vertical Sem Fio 2 em 1 Inova Cases 120W, Bivolt, com LED</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portáteis</t>
+          <t xml:space="preserve">Vertical</t>
         </is>
       </c>
       <c r="D30">
-        <v>289.0</v>
+        <v>428.0</v>
       </c>
       <c r="E30">
-        <v>208.9</v>
+        <v>290.61</v>
       </c>
       <c r="F30"/>
       <c r="G30" t="inlineStr">
@@ -1164,58 +1180,58 @@
       <c r="H30"/>
       <c r="I30"/>
       <c r="J30">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
+          <t xml:space="preserve">bloco de preço ML não encontrado</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lilin Aspirador de Pó Vertical Sem Fio i7 com Tubo Flexível 30000Pa Bivolt</t>
+          <t xml:space="preserve">Aspirador de Pó e Água JAGFOR 15L 3500W, para Sólidos e Líquidos, Casa, Carro e Oficina</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portáteis</t>
+          <t xml:space="preserve">Profissionais</t>
         </is>
       </c>
       <c r="D31">
-        <v>691.0</v>
+        <v>1299.0</v>
       </c>
       <c r="E31">
-        <v>656.0</v>
-      </c>
-      <c r="F31"/>
+        <v>435.53</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$1299.00 por R$435.53</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H31"/>
       <c r="I31"/>
       <c r="J31">
-        <v>4</v>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">preço não encontrado perto do buy-box (pode exigir JS / fora de estoque)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K31"/>
     </row>
     <row r="32">
       <c r="A32">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó Vertical com Fio Portátil 2 em 1 1300W Electrolux PTE10 220V</t>
+          <t xml:space="preserve">Dreame H60 GT, Aspirador Vertical Sem Fio Seco e Úmido, Sucção 21kPa, Reclinável 180°, Autolimpeza a 90°C, 220V-240V</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1224,84 +1240,96 @@
         </is>
       </c>
       <c r="D32">
-        <v>249.9</v>
+        <v>3299.0</v>
       </c>
       <c r="E32">
-        <v>208.9</v>
-      </c>
-      <c r="F32"/>
+        <v>2820.55</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$3299.00 por R$2969.00</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H32"/>
       <c r="I32"/>
       <c r="J32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">eufy C28 Robô Aspirador e Passa Pano, Esfregão Sempre Limpo, 15.000 Pa, 127V</t>
+          <t xml:space="preserve">Electrolux Aspirador de Pó e Água Hidrolux AWD01 1400W, 12L, Função Sopro, 127V</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Aspiradores</t>
         </is>
       </c>
       <c r="D33">
-        <v>6999.0</v>
+        <v>339.9</v>
       </c>
       <c r="E33">
-        <v>5984.14</v>
-      </c>
-      <c r="F33"/>
+        <v>157.4</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$339.90 por R$199.90</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
-        </is>
-      </c>
-      <c r="H33"/>
-      <c r="I33"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H33">
+        <v>339.9</v>
+      </c>
+      <c r="I33">
+        <v>199.9</v>
+      </c>
       <c r="J33">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lilin Robô Aspirador e Passa Pano X6 Mapeamento LiDAR 6500Pa 3 em 1 Bivolt</t>
+          <t xml:space="preserve">Britânia Aspirador de Pó Vertical 2 em 1 BAS1295P 1350W, Filtro HEPA, 127V (Oferta Amazon)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Vertical</t>
         </is>
       </c>
       <c r="D34">
-        <v>1519.0</v>
+        <v>204.0</v>
       </c>
       <c r="E34">
-        <v>1519.0</v>
+        <v>122.9</v>
       </c>
       <c r="F34"/>
       <c r="G34" t="inlineStr">
@@ -1316,103 +1344,111 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); fallback Tavily tentado mas não encontrou preço confiável</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrolux Aspirador de Pó com Saco Experience EQP40 1800W, Filtro HEPA, 127V</t>
+          <t xml:space="preserve">Electrolux Aspirador Vertical com Fio STK15, 2 em 1, 1450W, Filtro HEPA, 220V</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspiradores</t>
+          <t xml:space="preserve">Vertical</t>
         </is>
       </c>
       <c r="D35">
-        <v>849.0</v>
+        <v>319.9</v>
       </c>
       <c r="E35">
-        <v>474.02</v>
-      </c>
-      <c r="F35"/>
+        <v>189.9</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$319.90 por R$189.90</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H35"/>
       <c r="I35"/>
       <c r="J35">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrolux Aspirador Vertical com Fio STK15, 2 em 1, 1450W, Filtro HEPA, 220V</t>
+          <t xml:space="preserve">Electrolux Aspirador de Pó com Saco Experience EQP40 1800W, Filtro HEPA, 127V</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vertical</t>
+          <t xml:space="preserve">Aspiradores</t>
         </is>
       </c>
       <c r="D36">
-        <v>319.9</v>
+        <v>849.0</v>
       </c>
       <c r="E36">
-        <v>189.9</v>
-      </c>
-      <c r="F36"/>
+        <v>474.02</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$499.90 por R$499.90</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H36"/>
       <c r="I36"/>
       <c r="J36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Britânia Aspirador de Pó Vertical 2 em 1 BAS1295P 1350W, Filtro HEPA, 127V (Oferta Amazon)</t>
+          <t xml:space="preserve">Lilin Robô Aspirador e Passa Pano X6 Mapeamento LiDAR 6500Pa 3 em 1 Bivolt</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vertical</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D37">
-        <v>204.0</v>
+        <v>1519.0</v>
       </c>
       <c r="E37">
-        <v>122.9</v>
+        <v>1519.0</v>
       </c>
       <c r="F37"/>
       <c r="G37" t="inlineStr">
@@ -1427,54 +1463,58 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); fallback Tavily tentado mas não encontrou preço confiável</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrolux Aspirador de Pó e Água Hidrolux AWD01 1400W, 12L, Função Sopro, 127V</t>
+          <t xml:space="preserve">eufy C28 Robô Aspirador e Passa Pano, Esfregão Sempre Limpo, 15.000 Pa, 127V</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspiradores</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D38">
-        <v>339.9</v>
+        <v>6999.0</v>
       </c>
       <c r="E38">
-        <v>157.4</v>
-      </c>
-      <c r="F38"/>
+        <v>5984.14</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R$6999.00</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
-        </is>
-      </c>
-      <c r="H38"/>
-      <c r="I38"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H38">
+        <v>6999.0</v>
+      </c>
+      <c r="I38">
+        <v>6999.0</v>
+      </c>
       <c r="J38">
-        <v>7</v>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K38"/>
     </row>
     <row r="39">
       <c r="A39">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dreame H60 GT, Aspirador Vertical Sem Fio Seco e Úmido, Sucção 21kPa, Reclinável 180°, Autolimpeza a 90°C, 220V-240V</t>
+          <t xml:space="preserve">Aspirador de Pó Vertical com Fio Portátil 2 em 1 1300W Electrolux PTE10 220V</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1483,84 +1523,96 @@
         </is>
       </c>
       <c r="D39">
-        <v>3299.0</v>
+        <v>249.9</v>
       </c>
       <c r="E39">
-        <v>2820.55</v>
-      </c>
-      <c r="F39"/>
+        <v>208.9</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$209.90 por R$209.90</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H39"/>
       <c r="I39"/>
       <c r="J39">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó e Água JAGFOR 15L 3500W, para Sólidos e Líquidos, Casa, Carro e Oficina</t>
+          <t xml:space="preserve">Lilin Aspirador de Pó Vertical Sem Fio i7 com Tubo Flexível 30000Pa Bivolt</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Profissionais</t>
+          <t xml:space="preserve">Portáteis</t>
         </is>
       </c>
       <c r="D40">
+        <v>691.0</v>
+      </c>
+      <c r="E40">
+        <v>656.0</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$1299.00 por R$1299.00</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H40">
         <v>1299.0</v>
       </c>
-      <c r="E40">
-        <v>435.53</v>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">de R$1299.00 por R$435.53</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">correto</t>
-        </is>
-      </c>
-      <c r="H40"/>
-      <c r="I40"/>
+      <c r="I40">
+        <v>1299.0</v>
+      </c>
       <c r="J40">
         <v>0</v>
       </c>
-      <c r="K40"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">âncora do produto não encontrada; preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó Vertical Sem Fio 2 em 1 Inova Cases 120W, Bivolt, com LED</t>
+          <t xml:space="preserve">Black+Decker Aspirador de Pó e Água Portátil à Bateria 3,6V APB3600 Vermelho Bivolt</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vertical</t>
+          <t xml:space="preserve">Portáteis</t>
         </is>
       </c>
       <c r="D41">
-        <v>428.0</v>
+        <v>289.0</v>
       </c>
       <c r="E41">
-        <v>290.61</v>
+        <v>208.9</v>
       </c>
       <c r="F41"/>
       <c r="G41" t="inlineStr">
@@ -1571,21 +1623,21 @@
       <c r="H41"/>
       <c r="I41"/>
       <c r="J41">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t xml:space="preserve">não encontrou bloco de preço ML</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); fallback Tavily tentado mas não encontrou preço confiável</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó Vertical 2 em 1 Philco PAS1550C 1400W</t>
+          <t xml:space="preserve">WAP Aspirador de Pó Vertical à Bateria Eco Rápido 2 em 1, 700ml, Bivolt</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1594,14 +1646,14 @@
         </is>
       </c>
       <c r="D42">
-        <v>208.0</v>
+        <v>959.9</v>
       </c>
       <c r="E42">
-        <v>192.0</v>
+        <v>499.9</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$206.90 por R$159.82</t>
+          <t xml:space="preserve">de R$959.90 por R$699.90</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1610,162 +1662,162 @@
         </is>
       </c>
       <c r="H42">
-        <v>206.9</v>
+        <v>959.9</v>
       </c>
       <c r="I42">
-        <v>159.82</v>
+        <v>699.9</v>
       </c>
       <c r="J42">
         <v>0</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t xml:space="preserve">price_to 192.00 -&gt; 159.82</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó Mondial Turbo Cycle HEPA 1550W AP-41-GI</t>
+          <t xml:space="preserve">WAP Robô Aspirador de Pó ROBOT W90 3 em 1, Automático, 250ml, Bivolt</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vertical</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D43">
-        <v>329.9</v>
+        <v>359.9</v>
       </c>
       <c r="E43">
-        <v>235.47</v>
+        <v>315.76</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$329.90 por R$235.50</t>
+          <t xml:space="preserve">de R$549.90 por R$359.90</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">correto</t>
-        </is>
-      </c>
-      <c r="H43"/>
-      <c r="I43"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H43">
+        <v>549.9</v>
+      </c>
+      <c r="I43">
+        <v>359.9</v>
+      </c>
       <c r="J43">
         <v>0</v>
       </c>
-      <c r="K43"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó Sem Fio Arno X-Force Flex 9.60 RH20</t>
+          <t xml:space="preserve">WAP Aspirador de Pó e Água GTW Inox 70i 2800W com Autolimpeza e Bocal de Sopro 70 Litros 127V</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vertical</t>
+          <t xml:space="preserve">Profissionais</t>
         </is>
       </c>
       <c r="D44">
-        <v>1599.0</v>
+        <v>2099.9</v>
       </c>
       <c r="E44">
-        <v>999.0</v>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">de R$1599.00 por R$1199.00</t>
-        </is>
-      </c>
+        <v>1994.9</v>
+      </c>
+      <c r="F44"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">corrigido</t>
-        </is>
-      </c>
-      <c r="H44">
-        <v>1599.0</v>
-      </c>
-      <c r="I44">
-        <v>1199.0</v>
-      </c>
+          <t xml:space="preserve">não_verificado</t>
+        </is>
+      </c>
+      <c r="H44"/>
+      <c r="I44"/>
       <c r="J44">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t xml:space="preserve">price_to 999.00 -&gt; 1199.00</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); fallback Tavily tentado mas não encontrou preço confiável</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó Mondial Turbo Cycle AP-36 1100W, 2 em 1</t>
+          <t xml:space="preserve">Electrolux Aspirador de Pó e Água A10N1 1400W 18L (11L útil) com Função Sopro 127V</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vertical</t>
+          <t xml:space="preserve">Profissionais</t>
         </is>
       </c>
       <c r="D45">
-        <v>316.9</v>
+        <v>379.9</v>
       </c>
       <c r="E45">
-        <v>196.97</v>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">de R$316.90 por R$196.97</t>
-        </is>
-      </c>
+        <v>259.9</v>
+      </c>
+      <c r="F45"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">correto</t>
+          <t xml:space="preserve">não_verificado</t>
         </is>
       </c>
       <c r="H45"/>
       <c r="I45"/>
       <c r="J45">
-        <v>0</v>
-      </c>
-      <c r="K45"/>
+        <v>7</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); fallback Tavily tentado mas não encontrou preço confiável</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mini Aspirador de Pó Betahome Portátil 120W, USB, Soprador, Sem Fio, 6000Pa</t>
+          <t xml:space="preserve">Xiaomi Robô Aspirador de Pó Inteligente S40C Branco</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portáteis</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D46">
-        <v>61.76</v>
+        <v>2699.99</v>
       </c>
       <c r="E46">
-        <v>41.99</v>
+        <v>1055.0</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$61.76 por R$41.99</t>
+          <t xml:space="preserve">de R$2699.99 por R$1035.00</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -1778,31 +1830,35 @@
       <c r="J46">
         <v>0</v>
       </c>
-      <c r="K46"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pelos Kärcher Pet Clean com Tosador Recarregável, Kit 5 em 1, 300W</t>
+          <t xml:space="preserve">Xiaomi Robô Aspirador de Pó Inteligente S40 Branco</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portáteis</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D47">
-        <v>542.56</v>
+        <v>1290.0</v>
       </c>
       <c r="E47">
-        <v>542.56</v>
+        <v>1220.0</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$749.00 por R$534.31</t>
+          <t xml:space="preserve">de R$1240.00 por R$1240.00</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -1815,60 +1871,60 @@
       <c r="J47">
         <v>0</v>
       </c>
-      <c r="K47"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó Vertical Sem Fio 3 em 1 Oster OASP630</t>
+          <t xml:space="preserve">Aspirador de Pó Philco PAS70 1800W 2,2L Super Silencioso com Filtro HEPA 127V</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vertical</t>
+          <t xml:space="preserve">Aspiradores</t>
         </is>
       </c>
       <c r="D48">
-        <v>507.0</v>
+        <v>347.9</v>
       </c>
       <c r="E48">
-        <v>466.44</v>
+        <v>313.39</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$539.90 por R$334.22</t>
+          <t xml:space="preserve">de R$339.90 por R$339.90</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t xml:space="preserve">corrigido</t>
-        </is>
-      </c>
-      <c r="H48">
-        <v>539.9</v>
-      </c>
-      <c r="I48">
-        <v>334.22</v>
-      </c>
+          <t xml:space="preserve">correto</t>
+        </is>
+      </c>
+      <c r="H48"/>
+      <c r="I48"/>
       <c r="J48">
         <v>0</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t xml:space="preserve">price_to 466.44 -&gt; 334.22</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó Vertical e Portátil WAP High Speed Plus 1350W, Tecnologia Cyclone, Filtro HEPA, 3 em 1, Vermelho</t>
+          <t xml:space="preserve">Kärcher Aspirador de Pó Vertical 2 em 1 VCL 2 com Filtro HEPA 127V</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1877,14 +1933,14 @@
         </is>
       </c>
       <c r="D49">
-        <v>316.9</v>
+        <v>399.0</v>
       </c>
       <c r="E49">
-        <v>196.97</v>
+        <v>224.91</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$207.00 por R$144.53</t>
+          <t xml:space="preserve">de R$399.00 por R$249.90</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -1893,27 +1949,27 @@
         </is>
       </c>
       <c r="H49">
-        <v>207.0</v>
+        <v>399.0</v>
       </c>
       <c r="I49">
-        <v>144.53</v>
+        <v>249.9</v>
       </c>
       <c r="J49">
         <v>0</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t xml:space="preserve">price_to 196.97 -&gt; 144.53</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Britânia BAS1295P Aspirador de Pó 2 em 1 1250W Preto 127V</t>
+          <t xml:space="preserve">Electrolux Aspirador de Pó Vertical Ergorapido 2 em 1 ERG25N 38min Bivolt Azul</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1922,14 +1978,14 @@
         </is>
       </c>
       <c r="D50">
-        <v>185.36</v>
+        <v>1299.0</v>
       </c>
       <c r="E50">
-        <v>129.9</v>
+        <v>759.9</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$185.36 por R$129.90</t>
+          <t xml:space="preserve">de R$1299.00 por R$760.90</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -1942,52 +1998,64 @@
       <c r="J50">
         <v>0</v>
       </c>
-      <c r="K50"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robô Aspirador Liectroux T9 com Base Autolimpante, Aspira, Varre e Passa Pano, para Carpetes e Pelo de Animais</t>
+          <t xml:space="preserve">Electrolux Aspirador de Pó sem Saco Easybox Bocal Pet EAS41 1800W Filtro HEPA 220V</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Aspiradores</t>
         </is>
       </c>
       <c r="D51">
-        <v>2899.0</v>
+        <v>952.0</v>
       </c>
       <c r="E51">
-        <v>2413.0</v>
+        <v>661.93</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$2899.00 por R$2413.00</t>
+          <t xml:space="preserve">de R$952.00 por R$774.18</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t xml:space="preserve">correto</t>
-        </is>
-      </c>
-      <c r="H51"/>
-      <c r="I51"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H51">
+        <v>952.0</v>
+      </c>
+      <c r="I51">
+        <v>774.18</v>
+      </c>
       <c r="J51">
         <v>0</v>
       </c>
-      <c r="K51"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador Vertical WAP Power Speed Max AZ20 1600W, Sistema 360° com Tecnologia Cyclone, 3 em 1, 127V</t>
+          <t xml:space="preserve">Midea Aspirador de Pó Vertical 2 em 1 1350W Preto e Azul 220V</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1996,14 +2064,14 @@
         </is>
       </c>
       <c r="D52">
-        <v>359.9</v>
+        <v>209.0</v>
       </c>
       <c r="E52">
-        <v>237.9</v>
+        <v>141.45</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$359.90 por R$237.90</t>
+          <t xml:space="preserve">de R$209.00 por R$149.00</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2016,114 +2084,130 @@
       <c r="J52">
         <v>0</v>
       </c>
-      <c r="K52"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robô Aspirador Xiaomi S40 10.000Pa Ultra Potente Bivolt Branco</t>
+          <t xml:space="preserve">Philco Aspirador de Pó Vertical Power Clean PAS4000V 2000W 220V</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Vertical</t>
         </is>
       </c>
       <c r="D53">
-        <v>1209.0</v>
+        <v>434.9</v>
       </c>
       <c r="E53">
-        <v>1209.0</v>
+        <v>234.99</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$1188.00 por R$1128.00</t>
+          <t xml:space="preserve">de R$434.90 por R$201.90</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t xml:space="preserve">correto</t>
-        </is>
-      </c>
-      <c r="H53"/>
-      <c r="I53"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H53">
+        <v>434.9</v>
+      </c>
+      <c r="I53">
+        <v>201.9</v>
+      </c>
       <c r="J53">
         <v>0</v>
       </c>
-      <c r="K53"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó e Água Wap GTW Inox 12 1400W com Bocal de Sopro</t>
+          <t xml:space="preserve">WAP Robô Aspirador de Pó ROBOT W100 3 em 1, Automático, 250ml, Bivolt</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspiradores</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D54">
-        <v>485.57</v>
+        <v>799.9</v>
       </c>
       <c r="E54">
-        <v>260.91</v>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">de R$696.00 por R$283.51</t>
-        </is>
-      </c>
+        <v>648.87</v>
+      </c>
+      <c r="F54"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t xml:space="preserve">correto</t>
+          <t xml:space="preserve">não_verificado</t>
         </is>
       </c>
       <c r="H54"/>
       <c r="I54"/>
       <c r="J54">
-        <v>0</v>
-      </c>
-      <c r="K54"/>
+        <v>7</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">preço não encontrado na janela da âncora (provável renderização JS); fallback Tavily tentado mas não encontrou preço confiável</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robô Aspirador e Esfregão Combinado 3 em 1 com Sucção 6500Pa</t>
+          <t xml:space="preserve">Kärcher Aspirador WDL 1s 3 em 1 Pó, Água e Soprador 1700W Tanque Inox 110V</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Profissionais</t>
         </is>
       </c>
       <c r="D55">
-        <v>999.0</v>
+        <v>479.0</v>
       </c>
       <c r="E55">
-        <v>532.97</v>
+        <v>323.91</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$999.00 por R$532.97</t>
+          <t xml:space="preserve">R$479.00</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t xml:space="preserve">correto</t>
-        </is>
-      </c>
-      <c r="H55"/>
-      <c r="I55"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H55">
+        <v>479.0</v>
+      </c>
+      <c r="I55">
+        <v>479.0</v>
+      </c>
       <c r="J55">
         <v>0</v>
       </c>
@@ -2131,23 +2215,23 @@
     </row>
     <row r="56">
       <c r="A56">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dreame X50 Ultra Robô Aspirador e Esfregão, 20.000Pa, supera obstáculos de 6 cm, mopa extensível e removível, navegação LDS inteligente, 127V</t>
+          <t xml:space="preserve">Electrolux Aspirador de Pó Sem Saco Ease C4 EAS40 1600W Cyclonic Power Filtro HEPA 127V</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Aspiradores</t>
         </is>
       </c>
       <c r="D56">
-        <v>4749.0</v>
+        <v>729.9</v>
       </c>
       <c r="E56">
-        <v>4749.0</v>
+        <v>539.9</v>
       </c>
       <c r="F56"/>
       <c r="G56" t="inlineStr">
@@ -2158,74 +2242,78 @@
       <c r="H56"/>
       <c r="I56"/>
       <c r="J56">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t xml:space="preserve">bloqueado (página pequena)</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); fallback Tavily tentado mas não encontrou preço confiável</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57">
-        <v>13</v>
+        <v>56</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">WAP Aspirador de Pó e Água GTW INOX 20i, Compacto, 20 Litros, com Soprador e Filtro Lavável, 170mbar 1900W 220v</t>
+          <t xml:space="preserve">Philco Aspirador Robô PAS23 3 em 1 com MOP Bivolt Anticolisão</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Profissionais</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D57">
-        <v>759.9</v>
+        <v>699.9</v>
       </c>
       <c r="E57">
-        <v>500.47</v>
-      </c>
-      <c r="F57"/>
+        <v>484.4</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de R$699.90 por R$509.87</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t xml:space="preserve">não_verificado</t>
+          <t xml:space="preserve">correto</t>
         </is>
       </c>
       <c r="H57"/>
       <c r="I57"/>
       <c r="J57">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t xml:space="preserve">preço não encontrado perto do buy-box (pode exigir JS / fora de estoque)</t>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robô Aspirador WAP Robot W200 3 em 1 Varre, Aspira e Passa Pano Bivolt</t>
+          <t xml:space="preserve">Mondial Aspirador de Pó Hepa Turbo AP-15 1500W 110V</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Aspiradores</t>
         </is>
       </c>
       <c r="D58">
-        <v>699.9</v>
+        <v>439.9</v>
       </c>
       <c r="E58">
-        <v>559.0</v>
+        <v>246.05</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$999.00 por R$565.62</t>
+          <t xml:space="preserve">de R$259.00 por R$259.00</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2238,15 +2326,19 @@
       <c r="J58">
         <v>0</v>
       </c>
-      <c r="K58"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59">
-        <v>11</v>
+        <v>58</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó Vertical e Portátil WAP High Speed Plus 1350W 3 em 1</t>
+          <t xml:space="preserve">Electrolux Aspirador de Pó Vertical Ergorapido 2 em 1 ERG24N 30min Bivolt</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2255,51 +2347,59 @@
         </is>
       </c>
       <c r="D59">
-        <v>326.0</v>
+        <v>1099.99</v>
       </c>
       <c r="E59">
-        <v>164.99</v>
+        <v>759.0</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$326.00 por R$160.04</t>
+          <t xml:space="preserve">de R$979.90 por R$979.90</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t xml:space="preserve">correto</t>
-        </is>
-      </c>
-      <c r="H59"/>
-      <c r="I59"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H59">
+        <v>979.9</v>
+      </c>
+      <c r="I59">
+        <v>979.9</v>
+      </c>
       <c r="J59">
         <v>0</v>
       </c>
-      <c r="K59"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60">
-        <v>10</v>
+        <v>59</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mini Aspirador De Pó Portátil Recarregável Chrome Technology Soprador Usb Automotivo 3em1 Sem Fio</t>
+          <t xml:space="preserve">Britânia Aspirador de Pó Vertical BAS1500V Filtro Ciclone 1500W 220V</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portáteis</t>
+          <t xml:space="preserve">Vertical</t>
         </is>
       </c>
       <c r="D60">
-        <v>59.99</v>
+        <v>249.0</v>
       </c>
       <c r="E60">
-        <v>39.98</v>
+        <v>153.49</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$59.99 por R$37.61</t>
+          <t xml:space="preserve">de R$159.90 por R$147.90</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2312,31 +2412,35 @@
       <c r="J60">
         <v>0</v>
       </c>
-      <c r="K60"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
-        <v>9</v>
+        <v>60</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robô Aspirador Wap Robot W90 Varre, Aspira e Passa Pano 30W Preto</t>
+          <t xml:space="preserve">Philips Walita Aspirador de Pó Vertical com Mop Série 3000 XC3133/01</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Vertical</t>
         </is>
       </c>
       <c r="D61">
-        <v>514.14</v>
+        <v>1999.9</v>
       </c>
       <c r="E61">
-        <v>359.9</v>
+        <v>1329.91</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$514.14 por R$359.90</t>
+          <t xml:space="preserve">de R$1329.91 por R$1329.91</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2349,68 +2453,80 @@
       <c r="J61">
         <v>0</v>
       </c>
-      <c r="K61"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62">
-        <v>8</v>
+        <v>61</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador Vertical WAP POWER SPEED MAX CI10 3 EM 1 1600W 127V</t>
+          <t xml:space="preserve">Robô Aspirador de Pó X600 com Mapeamento a Laser 3000Pa e Passa Pano</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vertical</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D62">
-        <v>359.9</v>
+        <v>1048.19</v>
       </c>
       <c r="E62">
-        <v>226.73</v>
+        <v>1048.19</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$359.90 por R$237.90</t>
+          <t xml:space="preserve">de R$1199.00 por R$1199.00</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t xml:space="preserve">correto</t>
-        </is>
-      </c>
-      <c r="H62"/>
-      <c r="I62"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H62">
+        <v>1199.0</v>
+      </c>
+      <c r="I62">
+        <v>1199.0</v>
+      </c>
       <c r="J62">
         <v>0</v>
       </c>
-      <c r="K62"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63">
-        <v>7</v>
+        <v>62</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador De Pó Portátil 21v + Filtro Hepa Com Acessórios</t>
+          <t xml:space="preserve">Velds Robô Aspirador V50 PRO Base Autolimpante Mop Duplo Giratório 10000Pa 127V</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portáteis</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D63">
-        <v>699.04</v>
+        <v>2449.99</v>
       </c>
       <c r="E63">
-        <v>289.9</v>
+        <v>2327.49</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$699.04 por R$289.90</t>
+          <t xml:space="preserve">de R$2449.99 por R$2449.99</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2423,52 +2539,64 @@
       <c r="J63">
         <v>0</v>
       </c>
-      <c r="K63"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robô Aspirador De Pó Inteligente Passa Pano Mapeamento Ekaza Preto</t>
+          <t xml:space="preserve">Arno X-CLEAN 4 Limpadora de Pisos Vertical Sem Fio 2 em 1 LXC4 Bivolt</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Robôs</t>
+          <t xml:space="preserve">Vertical</t>
         </is>
       </c>
       <c r="D64">
-        <v>999.0</v>
+        <v>2849.04</v>
       </c>
       <c r="E64">
-        <v>565.62</v>
+        <v>2899.99</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$999.00 por R$565.62</t>
+          <t xml:space="preserve">de R$3799.00 por R$3799.00</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t xml:space="preserve">correto</t>
-        </is>
-      </c>
-      <c r="H64"/>
-      <c r="I64"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H64">
+        <v>3799.0</v>
+      </c>
+      <c r="I64">
+        <v>3799.0</v>
+      </c>
       <c r="J64">
         <v>0</v>
       </c>
-      <c r="K64"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador Portátil 3 Em 1 Com Soprador e Filtro HEPA Para Carro e Teclado USB</t>
+          <t xml:space="preserve">Arno X-FORCE FLEX 9.60 Aqua Aspirador Versátil Sem Fio com Tubo Flexível XF9A Bivolt</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2477,14 +2605,14 @@
         </is>
       </c>
       <c r="D65">
-        <v>59.99</v>
+        <v>1819.0</v>
       </c>
       <c r="E65">
-        <v>39.99</v>
+        <v>1249.99</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$59.99 por R$37.61</t>
+          <t xml:space="preserve">de R$1499.00 por R$1249.99</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2497,31 +2625,35 @@
       <c r="J65">
         <v>0</v>
       </c>
-      <c r="K65"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador de Pó e Água WAP GTW 10 1400W de Potência com Bocal de Sopro</t>
+          <t xml:space="preserve">Arno X-PERT 7.60 Aspirador Versátil Sem Fio Bateria Removível RH6A Bivolt</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspiradores</t>
+          <t xml:space="preserve">Portáteis</t>
         </is>
       </c>
       <c r="D66">
-        <v>485.57</v>
+        <v>719.28</v>
       </c>
       <c r="E66">
-        <v>257.9</v>
+        <v>698.99</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$485.57 por R$260.91</t>
+          <t xml:space="preserve">de R$735.79 por R$697.70</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2534,40 +2666,48 @@
       <c r="J66">
         <v>0</v>
       </c>
-      <c r="K66"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bloqueio/pagina pequena (3905 bytes); preço resolvido via fallback Tavily</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67">
-        <v>3</v>
+        <v>66</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirador Automotivo Portátil WAP CAR com Filtro HEPA e Cabo de 3,7m</t>
+          <t xml:space="preserve">Robô Aspirador de Pó 3 em 1 – Varre Aspira e Passa Pano com Lds Mapeamento Lydsto R1D Compatível com XiaoMi Home</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portáteis</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D67">
-        <v>111.0</v>
+        <v>3500.0</v>
       </c>
       <c r="E67">
-        <v>99.9</v>
+        <v>1217.7</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$111.00 por R$99.90</t>
+          <t xml:space="preserve">de R$2590.00 por R$2159.00</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t xml:space="preserve">correto</t>
-        </is>
-      </c>
-      <c r="H67"/>
-      <c r="I67"/>
+          <t xml:space="preserve">corrigido</t>
+        </is>
+      </c>
+      <c r="H67">
+        <v>2590.0</v>
+      </c>
+      <c r="I67">
+        <v>2159.0</v>
+      </c>
       <c r="J67">
         <v>0</v>
       </c>
@@ -2575,11 +2715,11 @@
     </row>
     <row r="68">
       <c r="A68">
-        <v>2</v>
+        <v>67</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dreame L40 Ultra Com Base E Mop 19000pa Branco 127v</t>
+          <t xml:space="preserve">Robô De Limpeza Wap Robot W500 Policleaner</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2588,14 +2728,14 @@
         </is>
       </c>
       <c r="D68">
-        <v>7499.0</v>
+        <v>1399.0</v>
       </c>
       <c r="E68">
-        <v>6599.0</v>
+        <v>800.91</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$7499.00 por R$5999.00</t>
+          <t xml:space="preserve">de R$1399.00 por R$782.91</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2612,27 +2752,27 @@
     </row>
     <row r="69">
       <c r="A69">
-        <v>1</v>
+        <v>68</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Extratora de Sujeira Portátil WAP Spot Cleaner W3 Borrifa Esfrega e Extrai 1450W de Potência e Bico de Autolimpeza</t>
+          <t xml:space="preserve">Robô Aspirador Anker eufy X10 Pro 4 em 1 Sucção 8000Pa IA Evita Obstáculos Mapeamento AI.Map 3.0 Lava Seca Esvazia Reabastece Água Escovas Antiembaraço Navegação Laser Limpeza Silenciosa Ideal Pet220V</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Extratoras</t>
+          <t xml:space="preserve">Robôs</t>
         </is>
       </c>
       <c r="D69">
-        <v>1011.0</v>
+        <v>7999.0</v>
       </c>
       <c r="E69">
-        <v>489.28</v>
+        <v>4849.0</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t xml:space="preserve">de R$1011.00 por R$526.11</t>
+          <t xml:space="preserve">de R$7999.00 por R$4749.00</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">

</xml_diff>